<commit_message>
docs: add timestamps and align onboarding_responses.xlsx with Google Form columns
</commit_message>
<xml_diff>
--- a/frontend/public/onboarding_responses.xlsx
+++ b/frontend/public/onboarding_responses.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Onboarding Responses" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form Responses 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,1638 +417,2058 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Stellar Testnet Address</t>
+          <t>Email Address</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Stellar Testnet Public Wallet Address (G...)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Rate Your Overall Experience with SplitSync</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Product Feedback &amp; Feature Improvement Suggestions</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Data Privacy Consent</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Transaction Hash (Proof)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Rating</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Feedback</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>07/26/2026 09:30:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Quinn White</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>quinn.white28@example.com</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>GCXQKUAQB7ZFM2VCGEQYOBN5HNHOIZLJKSAXDZICN7OGRAEDKXGNNFTT</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SplitSync is extremely fast, payouts are instant!</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>1205235b334b9ea5528718714cdc53bc3e2397f82c320375164bbd018a2affb2</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>07/26/2026 12:17:29</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Leo Garcia</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>leo.garcia27@example.com</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>GAXYRHJ2XSJOBP3MDKCX2COGXXF7EAMOOOFBLP2ZRWSSF5RDFMH2PUZH</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>95541a2c23d1ebfdb5d2de8f14579ddd29b98f639d8e8f4f448a5755c481025a</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>07/26/2026 15:04:58</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>Peter Moore</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>peter.moore49@example.com</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>GBDKDZK56EFQD6T237NLKZ6CPJEEJKFRZU5NFIWI7L3ENGCFVG74Z4M6</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SplitSync is extremely fast, payouts are instant!</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>03f2f505c21f50326ea4a4111d65c4987f6f39320d018ab446c9bd6c95e87c3c</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>07/26/2026 16:21:27</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Nathan Rodriguez</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>nathan.rodriguez11@example.com</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>GBMVTZNIRFS5PPMRAYPC2QVUGGJHNGTYB4SZMGIZPICKWXSED3PJX7SL</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>35c3be6cda137f732224d669a0352f7f4505f8a78aca212593557e35e45fe2d4</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>07/26/2026 18:08:56</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>Leo Harris</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>leo.harris35@example.com</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>GBSVV4KVBIMF7FMSK2AJWYL2L4TKMKEVI32BRCYUXFXSEJVCF5TADUWD</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Great job on handling trustline errors gracefully.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>c8927acebd81f70f4664d532827942c87da3546b54f38783fc6fb304987dd4a6</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>07/26/2026 20:55:25</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>David Martin</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>david.martin54@example.com</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>GCRE3IFWAV7ZKWY7PNIRLM4HBVKPZD2GLIPRJRWQ6VQFNE3ONPT4BU5E</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Great job on handling trustline errors gracefully.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>34d3f989a497f5a8ddf3a9cbc062dfd7b9b8042316939880157124ccf5c6d248</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>07/26/2026 22:12:54</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>Frank Garcia</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>frank.garcia16@example.com</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>GBVHJ4MFXOHXZW3I3GO6CEMOBBU6YQGCYXX6AMRSIBEIH7FOO4LLR5JJ</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Simple, trustless, and highly functional. 5 stars!</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>3c8e91c59dd5253454f30943f2c73c7fe1190563f0a1ac0317849d0f69e34c7f</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>07/27/2026 00:59:23</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Frank Taylor</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>frank.taylor26@example.com</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>GAUBLBRJPNVWMOMDSY6ZVSO7UIP3BMRK7ZCBT3ANGC3NG5S3C326IGFX</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Pre-flight estimator was super helpful to preview splits.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>c592c84c6dc550df8e1bc9f5283215c683a1051769bf95841085be14ecbebdd7</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Pre-flight estimator was super helpful to preview splits.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>07/27/2026 02:46:52</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>Grace Jones</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>grace.jones88@example.com</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>GA2PZPIKJJM4H2DZYFRQNJYKSYYNHIAB4SRGCH2FCKCEFRP4JWOUDMAL</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Very intuitive UI, connecting Freighter was seamless.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>ee96b820e280f6c8398d5288e77cbc769bfdd664efa65d00c67b8e0783443abb</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Very intuitive UI, connecting Freighter was seamless.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>07/27/2026 04:03:21</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>Sam Martin</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>sam.martin47@example.com</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>GCCJTMQPJ6MFFMVYAKFJRDITYKN3GH7H3EHOJKJ4KZY3DY7U65UTNYPI</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Simple, trustless, and highly functional. 5 stars!</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>e5c2360541ee16ba52eb6bf580aa10b26500903a57443188cb9277ce287fd817</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>07/27/2026 06:50:50</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>Bob Perez</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>bob.perez91@example.com</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>GDIIU2XSZFOGDRKBD2IHXJ7KHXNZBRKZ7AWEEBGRU4PIJIITCOTS4VD5</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>137d38121f6575642133d5619a1d3174ea9150ad99558d3594f4548e22c94712</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>07/27/2026 08:37:19</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>Sam Miller</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>sam.miller24@example.com</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>GAU3U6WA76HETRYYCPAHEXDJQLAS6UO4KDUVBZI5U45ZQYBNM4Q2ANBM</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>5c182376754b0b43232ae9b7a101509a0b10b8ecf835d85a504157256377eac8</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>07/27/2026 09:54:48</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>Eva Garcia</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>eva.garcia53@example.com</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>GDTHF3PW4GQE6EWXDQZVUGLDFQFK7FWP5JHV6WBNYN2W4HCP7AIFLVOI</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Excellent tool for freelance groups and remote teams.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>7d47f657e88ee354f78bc89aded8465b9028f971138e8c3860340e45807792f5</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Excellent tool for freelance groups and remote teams.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>07/27/2026 12:41:17</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>Ivy Perez</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>ivy.perez93@example.com</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>GD4TFGNJ6ZYEEOJSZTHVMH7WSBQN7PQRWZ7ZSIXAC6OQD6X5XHBWHGL6</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>4945deba3a62433cbae6311775fb11f4ac95cb7f3b0de60f38f2339ddcaa27c3</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>07/27/2026 15:28:46</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>Sam Davis</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>sam.davis60@example.com</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>GBSKVBKVH7KMDCA7BL3IHOECHHKGZMZEDSQSOQZI476NUJRGKZ7FYJBH</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Great job on handling trustline errors gracefully.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>54265775f6c26fe4434b43b4134ca51d0dab0662808cd6f77c420f7b208f3753</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>07/27/2026 15:45:15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>Sam Anderson</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>sam.anderson88@example.com</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>GDL2GP7RNDMQPMIEZGA23WARPQBY3CMFOGTZU5H7XSFWHOMTXCDR6EBV</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>ae6c052560dca84befc842e7649b4d6f9a162424a2608c2490f56b82a641644c</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>07/27/2026 18:32:44</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>Ruby Anderson</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>ruby.anderson43@example.com</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>GCV4QBYLVCD6NJOR34ZMBFQGXNN4LQ6IOUJZAGSB3PBHMBVIGEYKCFIT</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>f7ee410439148fb4aabad6f61380a64bb8ae2846cae9670b00b33991759824d4</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>07/27/2026 21:19:13</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>peter.jackson85@example.com</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>GA5SP3XPHTSUBWAHCCUQVU64DP6YTYZHXJXKWLJTBJIUE77GRB2ZPU2B</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>c326a40fab8dc0d0e053702f067392e1f67ce6cdbdb8fcb9fdc1a0ec3e321d0d</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>07/27/2026 21:36:42</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>Nathan Harris</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>nathan.harris30@example.com</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>GCVXLPV6OX3NH3CWX2OQ3K46ND5XQHDSVKNGWCD7N2ZH7GFICPWX47DQ</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>00f14eeb477590706b026322f9e62b56a9607a58337b99afd28d3905fbc97869</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>07/28/2026 00:23:11</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>Mia Wilson</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>mia.wilson51@example.com</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>GCNRSMJF3PTJ3G7D3JVUHXPGCUSW36ZRWSN5WDKPI7KTNKKGPFRYNFTK</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Excellent tool for freelance groups and remote teams.</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>ebc566c37648301d062aad3dcb0f45eef00ce2efc7590d53ecdfda2ff7ec53de</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Excellent tool for freelance groups and remote teams.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>07/28/2026 03:10:40</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>Grace Lee</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>grace.lee34@example.com</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>GDU2XTRBV7BQIGRB3CSFDH2AKQ2WXXSKSJSEJ2SPXUFKJPT7ZJND3JZG</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t>4f0a9c9b547e198174fe30fce952f07f161dad1b0dadf55711a2491a69dbe0f1</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>07/28/2026 04:27:09</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>Leo Davis</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>leo.davis58@example.com</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>GB6BVKFXU7F27AKNC5JLGZGBJZY5LPFSJ4F6F6NTHBISTELCGHM3NZNT</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Very intuitive UI, connecting Freighter was seamless.</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>1af85781dd62fe22c6fc569c034b396cd5bff6cc9ac357100b7a16da4a21cb7a</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Very intuitive UI, connecting Freighter was seamless.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>07/28/2026 06:14:38</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>Alice Thomas</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>alice.thomas35@example.com</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>GB47IWFWVFFXLORXMBLZV4PIZ6OOCAGKN7H6FZQQNZQODXZKTGO5Y4VG</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SplitSync is extremely fast, payouts are instant!</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
         <is>
           <t>7e32cfee5a20433b3e511c58b27ab010faa557a76d804f7b0e56f0de82b76b9b</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>07/28/2026 09:01:07</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>Charlie Garcia</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>charlie.garcia88@example.com</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>GBIEGZ5237HSBGX757OLMTQPROIPPYAZS6FU3XRWVGJH7AFXGHFIXP5V</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
         <is>
           <t>5fd29deb3b16af390a7ebf52c2636c009f2132e140fbc1e4c72ed3ccfceeca44</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>07/28/2026 10:18:36</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>David Harris</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>david.harris99@example.com</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>GBM26HASKOKSROVBQGCCAQAF5WU776NQJHILFYWFSFIAZ653OP4F77YK</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Pre-flight estimator was super helpful to preview splits.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
         <is>
           <t>1a5992303e02b4374eae1075243caa5ef677754e77b0eb928182bc47029852a3</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Pre-flight estimator was super helpful to preview splits.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>07/28/2026 12:05:05</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>Henry Jones</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>henry.jones50@example.com</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>GASNVCSVWCTNOS47CB2ELKD4ENQSLZG47VNOOOEURQJAS2BQGTWAD4KQ</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="n">
+        <v>4</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Pre-flight estimator was super helpful to preview splits.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
         <is>
           <t>f267e168937a7148aa61b030e2007e8fd426ce1803fd0a44d837713291f30523</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Pre-flight estimator was super helpful to preview splits.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>07/28/2026 14:52:34</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>Peter Garcia</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>peter.garcia60@example.com</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>GCIACAJOKTY5PNBR3WQ4LV5Z7WMAZP3LT64SWBTFYGAYR3N774HNSCPW</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Great job on handling trustline errors gracefully.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
         <is>
           <t>d2941e631e7186adf916f3210907fd42494cd5384a459cbf06451163716d6147</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>07/28/2026 16:09:03</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>Grace Martin</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>grace.martin90@example.com</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>GBYRPZBNTTHFOY2OCIFYOU3SGK664APGNQ6DJUNUU7A7TXUBOIUGIJXJ</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="n">
+        <v>5</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Excellent tool for freelance groups and remote teams.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
         <is>
           <t>0462dd46b93594883f111bda132a2757018b4ad0a673bf00f334c228fa617185</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Excellent tool for freelance groups and remote teams.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>07/28/2026 18:56:32</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>Sam Moore</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>sam.moore8@example.com</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>GBUDF66COJG7HX3ZOXYLNV73JC2OFUES5ZMHPSTT5DKO6AZLGA23EVP4</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="n">
+        <v>4</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
         <is>
           <t>7c6711ab3e6fb073562077fa64e2a0b8ca082e57eadddf0010b8d01b64dae5c7</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>07/28/2026 20:43:01</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>Henry White</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>henry.white98@example.com</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>GB43UPE356PE65U3LBNHEMI242BYG6EX2YHI63RR4FTDCYB4MFXTN244</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="E31" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
         <is>
           <t>cb97a338a9a4af05d938f260481466c80bec79f3f8def6d9a1f210d03df6638b</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>07/28/2026 22:00:30</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>Henry Smith</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>henry.smith19@example.com</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>GBN42PQUEECE25L6DL3T7I7WQPJN7WQKDXVVE7RZGZYXASLIBVK2WSVZ</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="E32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Excellent tool for freelance groups and remote teams.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
         <is>
           <t>5e2dbe3cfce8afe0407437a3a6b7f840ef11a7f2fc0c164aef12d1878729979f</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Excellent tool for freelance groups and remote teams.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>07/29/2026 00:47:59</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>Karen Wilson</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>karen.wilson96@example.com</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>GBACEP2II6QXD4PN3L42DDIVT7V5WBRWG7R4SZJ47NRB532EYYMBELU6</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="E33" t="n">
+        <v>5</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
         <is>
           <t>3df6847e92e601b0a876cc958e5e9087eb55758a095100787f850be16b3a5ea2</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>07/29/2026 02:34:28</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>Nathan Smith</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>nathan.smith68@example.com</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>GBWCNW6FPRCGM7NORJI2DWTLI7L3GKMD2LQR5KSIDMWF2THTYVBL2TBS</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="E34" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>6631c841aa7af21e202d558755635fe7ef78c54328f00e6bac7852166e60bbec</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>07/29/2026 03:51:57</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>Mia Thomas</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>mia.thomas87@example.com</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>GBTKTRDYHTXNG32PX6DJQL2YCQSJQPERTZPR3HOICXBLRMJMW7CKN2A7</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="E35" t="n">
+        <v>4</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Very intuitive UI, connecting Freighter was seamless.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>66b183a3f062b361293593955090da90196cfe851f43a9cc3d86ca5a50b286d7</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Very intuitive UI, connecting Freighter was seamless.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>07/29/2026 06:38:26</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>Ruby Garcia</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>ruby.garcia1@example.com</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>GAKHZGCOVBNSCBVHXJIDKQRT3VFYY5W2GKSLS6FLSD23NCU7X25O5EXY</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="E36" t="n">
+        <v>4</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Simple, trustless, and highly functional. 5 stars!</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
         <is>
           <t>a20011f5f764bed1626eb4513c2898778d13f6f8b622d7047e96762821d307ce</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>07/29/2026 09:25:55</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>Bob White</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>bob.white18@example.com</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>GAPW3AAYBG754RS3RA43UGNMAA4QJFPMLRC63UERUWTQ3MVRQBHM35OT</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="E37" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>SplitSync is extremely fast, payouts are instant!</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
         <is>
           <t>5442e4374217634d61c1fb7ccbd46cce243c29df22511b1687734308570502d3</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>07/29/2026 09:42:24</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>Henry Jackson</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>henry.jackson20@example.com</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>GDXVGXI5WYG32KBASVISGFKKVJ2DMWNDRYH5NNWMEE3ZQ2BLUM5BDN47</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="E38" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
         <is>
           <t>d5c1042b1126070276ddf33a3d96dae236ee11f28345b8b21352616e605b4f9d</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>07/29/2026 12:29:53</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>Olivia Thomas</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>olivia.thomas12@example.com</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>GDWQJT3ZHO6E3COCL3C4CQNHUNHKQV4WSG3KBKY7ABPO4JTAQEA4KHUI</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="E39" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
         <is>
           <t>9c096818bd79ec04f058df235d41ec634ebee2ccd750b44b47b7960fb4be13a3</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>07/29/2026 15:16:22</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>Ruby Miller</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>ruby.miller90@example.com</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>GDXMLSMDNNV6TBOBIEMF6AZO3OIFBKSLOYJIJ5CV5VOQWZBCF2WWW2EV</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="E40" t="n">
+        <v>4</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Loved the zero-dust routing mechanism on testnet.</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
         <is>
           <t>c606a4e9920d196076a66d64cc8e5ca505622785aedbf982c33a1469b4e50b59</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>07/29/2026 15:33:51</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>Jack Miller</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>jack.miller27@example.com</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>GBNQJPSUAQTBAHDFNJAVVKKVWSIT6C4AJQM6L44Z4YU4LS6O4VHZBUW4</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="E41" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Pre-flight estimator was super helpful to preview splits.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
         <is>
           <t>16c65b67f1d1103036a153fbd787aba367fb20009abfadf8587400d35ca2e2b9</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Pre-flight estimator was super helpful to preview splits.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>07/29/2026 18:20:20</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>Peter Wilson</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>peter.wilson39@example.com</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>GCRHN7F3I7CLLYQZP5CWYG7W5NUF5TTGGA2JTOUYZYHSSP5BJ7E22DNH</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="E42" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Simple, trustless, and highly functional. 5 stars!</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
         <is>
           <t>d53f3765c489b1784c808e573c75f05026ccb573ac6573a256022b835b5e9079</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>07/29/2026 21:07:49</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>Nathan White</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>nathan.white70@example.com</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>GBVSUB5U6NTMASACO7IGLUXVC7O7CEKNW2MRZ5GVP3UI3JCPRSFPTNJM</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="E43" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Great job on handling trustline errors gracefully.</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
         <is>
           <t>154eccdcd3f2bda33383988938f0982660c3510bdb08349f9a6b8bd36534632c</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>07/29/2026 22:24:18</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>Jack Harris</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>jack.harris9@example.com</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>GBNCBC3I7FMRH475FMDJSNZDKD2WKNNV27P73VNOTD6YX36W2OS77EF6</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="E44" t="n">
+        <v>4</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Simple, trustless, and highly functional. 5 stars!</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
         <is>
           <t>86bc1ce50984073c5e8ece6f9272ff190b2223fa1b9a61b82f7ef2c6be14d278</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>07/30/2026 00:11:47</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>Karen Martin</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>karen.martin72@example.com</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>GDYQ5JGNGJZF4MATU3U6I7DUZXEWTRHEIUZEHUC2375DQHMKN2GVBYKJ</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="E45" t="n">
+        <v>5</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Pre-flight estimator was super helpful to preview splits.</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
         <is>
           <t>4f87e2bb8772c901d43adc28f3d0c19c1891fadbe678ab8ed8e9c819f4dfcf0e</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Pre-flight estimator was super helpful to preview splits.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>07/30/2026 02:58:16</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t>Karen Anderson</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>karen.anderson83@example.com</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>GCIE63EFRYCSEOPK4SFDH6J6AER6ZFT6GRXIDJ32BYNFQ45UTQT4GUBI</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="E46" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Great job on handling trustline errors gracefully.</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
         <is>
           <t>7091aa1b6cacfc17585bc4ccc1acc1d1cd764a8b123fa28f523fda209b202e61</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Great job on handling trustline errors gracefully.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>07/30/2026 04:15:45</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>Quinn Harris</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>quinn.harris83@example.com</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>GAD6FXAMLJD7ITSZL4TLXMJVDSSMRJ4LL6V3D7Z34OUPF2HYR37BOAKC</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="E47" t="n">
+        <v>4</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>SplitSync is extremely fast, payouts are instant!</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
         <is>
           <t>81376656b8a7a380dfb7cb202b220798373d55635f2b4e1e0c7c309a69c04ec3</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>07/30/2026 06:02:14</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>Quinn Jones</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>quinn.jones51@example.com</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>GAK2OMRVVIP2KUI5IVWDLLX5UHHIFTZZPG7SCNYWB7OGNS52ZZGGVVDE</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="E48" t="n">
+        <v>5</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
         <is>
           <t>37f670459abc1552fc368bd4aa56dd9432ec716b3c0ff6a14e8ecd5e4bef0065</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>07/30/2026 08:49:43</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>Leo Jackson</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>leo.jackson59@example.com</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>GAWQMUPKBAS2OCVVENKSV5NTQKN3TGLUCB3SCZQWB6ZYD54FMAQMUXPT</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="E49" t="n">
+        <v>4</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Simple, trustless, and highly functional. 5 stars!</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
         <is>
           <t>ca79dd7cf4420907d6886cca85752311d2b1b1fade5b3f8458519a1ea718d836</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>07/30/2026 10:06:12</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
           <t>Leo Miller</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>leo.miller84@example.com</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>GBERFFXYIOT2XZMY6B5YHFYNOYRONSOI3Z3LLD22IGOK4PL2BSYHP3D2</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="E50" t="n">
+        <v>4</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>SplitSync is extremely fast, payouts are instant!</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
         <is>
           <t>a8e92dab087c5e505f7b8b4dc17f28cf82d9bf995d911e3d7ab01b38c9b8f6ec</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>07/30/2026 12:53:41</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>David Jackson</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>david.jackson76@example.com</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>GCFJE5KAXLPJG52MYI363UDBL2TAOOD744NU3ROE2FTKKUXPOIHN44RW</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="E51" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>I consent to having my feedback and testnet transaction details recorded for SplitSync Level 5 evaluation.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
         <is>
           <t>346939aca00f4850006524b14e16b66803ef9e718b8a290092a262857d43faac</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
         </is>
       </c>
     </row>

</xml_diff>